<commit_message>
chore(ops): external-share sanitize, CentOS deploy, and demo samples
Remove real business samples and SDD/tmp artifacts; add external-share docs,
audit/prepare scripts, synthetic demo CSVs, Linux Compose overrides, and
require env for Feishu table IDs. Sanitize ops docs and blueprint push scripts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/samples/fob/01-volume-ed.xlsx
+++ b/docs/samples/fob/01-volume-ed.xlsx
@@ -441,10 +441,10 @@
         <v>3.37</v>
       </c>
       <c r="E3" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F3" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G3" t="str">
         <v>FOB</v>
@@ -464,10 +464,10 @@
         <v>4.52</v>
       </c>
       <c r="E4" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F4" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G4" t="str">
         <v>非退税</v>
@@ -487,10 +487,10 @@
         <v>4.52</v>
       </c>
       <c r="E5" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F5" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G5" t="str">
         <v>FOB</v>
@@ -510,10 +510,10 @@
         <v>4.52</v>
       </c>
       <c r="E6" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F6" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G6" t="str">
         <v>FOB</v>
@@ -533,10 +533,10 @@
         <v>5.67</v>
       </c>
       <c r="E7" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F7" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G7" t="str">
         <v>退税</v>
@@ -556,10 +556,10 @@
         <v>5.67</v>
       </c>
       <c r="E8" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F8" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G8" t="str">
         <v>FOB</v>
@@ -579,10 +579,10 @@
         <v>6.82</v>
       </c>
       <c r="E9" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F9" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G9" t="str">
         <v>退税</v>
@@ -602,10 +602,10 @@
         <v>6.82</v>
       </c>
       <c r="E10" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F10" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G10" t="str">
         <v>FOB</v>
@@ -625,10 +625,10 @@
         <v>7.97</v>
       </c>
       <c r="E11" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F11" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G11" t="str">
         <v>非退税</v>
@@ -648,10 +648,10 @@
         <v>7.97</v>
       </c>
       <c r="E12" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F12" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G12" t="str">
         <v>FOB</v>
@@ -671,10 +671,10 @@
         <v>9.12</v>
       </c>
       <c r="E13" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F13" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G13" t="str">
         <v>退税</v>
@@ -694,10 +694,10 @@
         <v>9.12</v>
       </c>
       <c r="E14" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F14" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G14" t="str">
         <v>FOB</v>
@@ -717,10 +717,10 @@
         <v>10.27</v>
       </c>
       <c r="E15" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F15" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G15" t="str">
         <v>退税</v>
@@ -740,10 +740,10 @@
         <v>10.27</v>
       </c>
       <c r="E16" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F16" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G16" t="str">
         <v>FOB</v>
@@ -763,10 +763,10 @@
         <v>10.27</v>
       </c>
       <c r="E17" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F17" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G17" t="str">
         <v>FOB</v>
@@ -786,10 +786,10 @@
         <v>3.37</v>
       </c>
       <c r="E18" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F18" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G18" t="str">
         <v>非退税</v>
@@ -809,10 +809,10 @@
         <v>3.37</v>
       </c>
       <c r="E19" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F19" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G19" t="str">
         <v>FOB</v>
@@ -832,10 +832,10 @@
         <v>4.52</v>
       </c>
       <c r="E20" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F20" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G20" t="str">
         <v>退税</v>
@@ -855,10 +855,10 @@
         <v>4.52</v>
       </c>
       <c r="E21" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F21" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G21" t="str">
         <v>FOB</v>
@@ -878,10 +878,10 @@
         <v>5.67</v>
       </c>
       <c r="E22" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F22" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G22" t="str">
         <v>退税</v>
@@ -901,10 +901,10 @@
         <v>5.67</v>
       </c>
       <c r="E23" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F23" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G23" t="str">
         <v>FOB</v>
@@ -924,10 +924,10 @@
         <v>6.82</v>
       </c>
       <c r="E24" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F24" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G24" t="str">
         <v>非退税</v>
@@ -947,10 +947,10 @@
         <v>6.82</v>
       </c>
       <c r="E25" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F25" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G25" t="str">
         <v>FOB</v>
@@ -970,10 +970,10 @@
         <v>7.97</v>
       </c>
       <c r="E26" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F26" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G26" t="str">
         <v>退税</v>
@@ -993,10 +993,10 @@
         <v>7.97</v>
       </c>
       <c r="E27" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F27" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G27" t="str">
         <v>FOB</v>
@@ -1016,10 +1016,10 @@
         <v>7.97</v>
       </c>
       <c r="E28" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F28" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G28" t="str">
         <v>FOB</v>
@@ -1039,10 +1039,10 @@
         <v>9.12</v>
       </c>
       <c r="E29" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F29" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G29" t="str">
         <v>退税</v>
@@ -1062,10 +1062,10 @@
         <v>9.12</v>
       </c>
       <c r="E30" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F30" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G30" t="str">
         <v>FOB</v>
@@ -1085,10 +1085,10 @@
         <v>10.27</v>
       </c>
       <c r="E31" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F31" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G31" t="str">
         <v>非退税</v>
@@ -1108,10 +1108,10 @@
         <v>10.27</v>
       </c>
       <c r="E32" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F32" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G32" t="str">
         <v>FOB</v>
@@ -1131,10 +1131,10 @@
         <v>3.37</v>
       </c>
       <c r="E33" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F33" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G33" t="str">
         <v>退税</v>
@@ -1154,10 +1154,10 @@
         <v>3.37</v>
       </c>
       <c r="E34" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F34" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G34" t="str">
         <v>FOB</v>
@@ -1177,10 +1177,10 @@
         <v>4.52</v>
       </c>
       <c r="E35" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F35" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G35" t="str">
         <v>退税</v>
@@ -1200,10 +1200,10 @@
         <v>4.52</v>
       </c>
       <c r="E36" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F36" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G36" t="str">
         <v>FOB</v>
@@ -1223,10 +1223,10 @@
         <v>5.67</v>
       </c>
       <c r="E37" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F37" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G37" t="str">
         <v>非退税</v>
@@ -1246,10 +1246,10 @@
         <v>5.67</v>
       </c>
       <c r="E38" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F38" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G38" t="str">
         <v>FOB</v>
@@ -1269,10 +1269,10 @@
         <v>5.67</v>
       </c>
       <c r="E39" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F39" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G39" t="str">
         <v>FOB</v>
@@ -1292,10 +1292,10 @@
         <v>6.82</v>
       </c>
       <c r="E40" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F40" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G40" t="str">
         <v>退税</v>
@@ -1315,10 +1315,10 @@
         <v>6.82</v>
       </c>
       <c r="E41" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F41" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G41" t="str">
         <v>FOB</v>
@@ -1338,10 +1338,10 @@
         <v>7.97</v>
       </c>
       <c r="E42" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F42" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G42" t="str">
         <v>退税</v>
@@ -1361,10 +1361,10 @@
         <v>7.97</v>
       </c>
       <c r="E43" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F43" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G43" t="str">
         <v>FOB</v>
@@ -1384,10 +1384,10 @@
         <v>9.12</v>
       </c>
       <c r="E44" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F44" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G44" t="str">
         <v>非退税</v>
@@ -1407,10 +1407,10 @@
         <v>9.12</v>
       </c>
       <c r="E45" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F45" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G45" t="str">
         <v>FOB</v>
@@ -1430,10 +1430,10 @@
         <v>10.27</v>
       </c>
       <c r="E46" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F46" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G46" t="str">
         <v>退税</v>
@@ -1453,10 +1453,10 @@
         <v>10.27</v>
       </c>
       <c r="E47" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F47" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G47" t="str">
         <v>FOB</v>
@@ -1476,10 +1476,10 @@
         <v>3.37</v>
       </c>
       <c r="E48" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F48" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G48" t="str">
         <v>退税</v>
@@ -1499,10 +1499,10 @@
         <v>3.37</v>
       </c>
       <c r="E49" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F49" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G49" t="str">
         <v>FOB</v>
@@ -1522,10 +1522,10 @@
         <v>3.37</v>
       </c>
       <c r="E50" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F50" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G50" t="str">
         <v>FOB</v>
@@ -1545,10 +1545,10 @@
         <v>4.52</v>
       </c>
       <c r="E51" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F51" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G51" t="str">
         <v>非退税</v>
@@ -1568,10 +1568,10 @@
         <v>4.52</v>
       </c>
       <c r="E52" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F52" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G52" t="str">
         <v>FOB</v>
@@ -1591,10 +1591,10 @@
         <v>5.67</v>
       </c>
       <c r="E53" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F53" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G53" t="str">
         <v>退税</v>
@@ -1614,10 +1614,10 @@
         <v>5.67</v>
       </c>
       <c r="E54" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F54" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G54" t="str">
         <v>FOB</v>
@@ -1637,10 +1637,10 @@
         <v>6.82</v>
       </c>
       <c r="E55" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F55" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G55" t="str">
         <v>退税</v>
@@ -1660,10 +1660,10 @@
         <v>6.82</v>
       </c>
       <c r="E56" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F56" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G56" t="str">
         <v>FOB</v>
@@ -1683,10 +1683,10 @@
         <v>7.97</v>
       </c>
       <c r="E57" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F57" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G57" t="str">
         <v>非退税</v>
@@ -1706,10 +1706,10 @@
         <v>7.97</v>
       </c>
       <c r="E58" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F58" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G58" t="str">
         <v>FOB</v>
@@ -1729,10 +1729,10 @@
         <v>9.12</v>
       </c>
       <c r="E59" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F59" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G59" t="str">
         <v>退税</v>
@@ -1752,10 +1752,10 @@
         <v>9.12</v>
       </c>
       <c r="E60" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F60" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G60" t="str">
         <v>FOB</v>
@@ -1775,10 +1775,10 @@
         <v>9.12</v>
       </c>
       <c r="E61" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F61" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G61" t="str">
         <v>FOB</v>
@@ -1798,10 +1798,10 @@
         <v>10.27</v>
       </c>
       <c r="E62" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F62" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G62" t="str">
         <v>退税</v>
@@ -1821,10 +1821,10 @@
         <v>10.27</v>
       </c>
       <c r="E63" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F63" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G63" t="str">
         <v>FOB</v>
@@ -1844,10 +1844,10 @@
         <v>3.37</v>
       </c>
       <c r="E64" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F64" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G64" t="str">
         <v>非退税</v>
@@ -1867,10 +1867,10 @@
         <v>3.37</v>
       </c>
       <c r="E65" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F65" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G65" t="str">
         <v>FOB</v>
@@ -1890,10 +1890,10 @@
         <v>4.52</v>
       </c>
       <c r="E66" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F66" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G66" t="str">
         <v>退税</v>
@@ -1913,10 +1913,10 @@
         <v>4.52</v>
       </c>
       <c r="E67" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F67" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G67" t="str">
         <v>FOB</v>
@@ -1936,10 +1936,10 @@
         <v>5.67</v>
       </c>
       <c r="E68" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F68" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G68" t="str">
         <v>退税</v>
@@ -1959,10 +1959,10 @@
         <v>5.67</v>
       </c>
       <c r="E69" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F69" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G69" t="str">
         <v>FOB</v>
@@ -1982,10 +1982,10 @@
         <v>6.82</v>
       </c>
       <c r="E70" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F70" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G70" t="str">
         <v>非退税</v>
@@ -2005,10 +2005,10 @@
         <v>6.82</v>
       </c>
       <c r="E71" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F71" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G71" t="str">
         <v>FOB</v>
@@ -2028,10 +2028,10 @@
         <v>6.82</v>
       </c>
       <c r="E72" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F72" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G72" t="str">
         <v>FOB</v>
@@ -2051,10 +2051,10 @@
         <v>7.97</v>
       </c>
       <c r="E73" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F73" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G73" t="str">
         <v>退税</v>
@@ -2074,10 +2074,10 @@
         <v>7.97</v>
       </c>
       <c r="E74" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F74" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G74" t="str">
         <v>FOB</v>
@@ -2097,10 +2097,10 @@
         <v>9.12</v>
       </c>
       <c r="E75" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F75" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G75" t="str">
         <v>退税</v>
@@ -2120,10 +2120,10 @@
         <v>9.12</v>
       </c>
       <c r="E76" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F76" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G76" t="str">
         <v>FOB</v>
@@ -2143,10 +2143,10 @@
         <v>10.27</v>
       </c>
       <c r="E77" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F77" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G77" t="str">
         <v>非退税</v>
@@ -2166,10 +2166,10 @@
         <v>10.27</v>
       </c>
       <c r="E78" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F78" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G78" t="str">
         <v>FOB</v>
@@ -2189,10 +2189,10 @@
         <v>3.37</v>
       </c>
       <c r="E79" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F79" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G79" t="str">
         <v>退税</v>
@@ -2212,10 +2212,10 @@
         <v>3.37</v>
       </c>
       <c r="E80" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F80" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G80" t="str">
         <v>FOB</v>
@@ -2235,10 +2235,10 @@
         <v>4.52</v>
       </c>
       <c r="E81" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F81" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G81" t="str">
         <v>退税</v>
@@ -2258,10 +2258,10 @@
         <v>4.52</v>
       </c>
       <c r="E82" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F82" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G82" t="str">
         <v>FOB</v>
@@ -2281,10 +2281,10 @@
         <v>4.52</v>
       </c>
       <c r="E83" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F83" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G83" t="str">
         <v>FOB</v>
@@ -2304,10 +2304,10 @@
         <v>5.67</v>
       </c>
       <c r="E84" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F84" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G84" t="str">
         <v>非退税</v>
@@ -2327,10 +2327,10 @@
         <v>5.67</v>
       </c>
       <c r="E85" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F85" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G85" t="str">
         <v>FOB</v>
@@ -2350,10 +2350,10 @@
         <v>6.82</v>
       </c>
       <c r="E86" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F86" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G86" t="str">
         <v>退税</v>
@@ -2373,10 +2373,10 @@
         <v>6.82</v>
       </c>
       <c r="E87" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F87" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G87" t="str">
         <v>FOB</v>
@@ -2396,10 +2396,10 @@
         <v>7.97</v>
       </c>
       <c r="E88" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F88" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G88" t="str">
         <v>退税</v>
@@ -2419,10 +2419,10 @@
         <v>7.97</v>
       </c>
       <c r="E89" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F89" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G89" t="str">
         <v>FOB</v>
@@ -2442,10 +2442,10 @@
         <v>9.12</v>
       </c>
       <c r="E90" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F90" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G90" t="str">
         <v>非退税</v>
@@ -2465,10 +2465,10 @@
         <v>9.12</v>
       </c>
       <c r="E91" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F91" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G91" t="str">
         <v>FOB</v>
@@ -2488,10 +2488,10 @@
         <v>10.27</v>
       </c>
       <c r="E92" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F92" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G92" t="str">
         <v>退税</v>
@@ -2511,10 +2511,10 @@
         <v>10.27</v>
       </c>
       <c r="E93" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F93" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G93" t="str">
         <v>FOB</v>
@@ -2534,10 +2534,10 @@
         <v>10.27</v>
       </c>
       <c r="E94" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F94" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G94" t="str">
         <v>FOB</v>
@@ -2557,10 +2557,10 @@
         <v>3.37</v>
       </c>
       <c r="E95" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F95" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G95" t="str">
         <v>退税</v>
@@ -2580,10 +2580,10 @@
         <v>3.37</v>
       </c>
       <c r="E96" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F96" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G96" t="str">
         <v>FOB</v>
@@ -2603,10 +2603,10 @@
         <v>4.52</v>
       </c>
       <c r="E97" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F97" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G97" t="str">
         <v>非退税</v>
@@ -2626,10 +2626,10 @@
         <v>4.52</v>
       </c>
       <c r="E98" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F98" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G98" t="str">
         <v>FOB</v>
@@ -2649,10 +2649,10 @@
         <v>5.67</v>
       </c>
       <c r="E99" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F99" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G99" t="str">
         <v>退税</v>
@@ -2672,10 +2672,10 @@
         <v>5.67</v>
       </c>
       <c r="E100" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F100" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G100" t="str">
         <v>FOB</v>
@@ -2695,10 +2695,10 @@
         <v>6.82</v>
       </c>
       <c r="E101" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F101" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G101" t="str">
         <v>退税</v>
@@ -2718,10 +2718,10 @@
         <v>6.82</v>
       </c>
       <c r="E102" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F102" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G102" t="str">
         <v>FOB</v>
@@ -2741,10 +2741,10 @@
         <v>7.97</v>
       </c>
       <c r="E103" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F103" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G103" t="str">
         <v>非退税</v>
@@ -2764,10 +2764,10 @@
         <v>7.97</v>
       </c>
       <c r="E104" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F104" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G104" t="str">
         <v>FOB</v>
@@ -2787,10 +2787,10 @@
         <v>7.97</v>
       </c>
       <c r="E105" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F105" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G105" t="str">
         <v>FOB</v>
@@ -2810,10 +2810,10 @@
         <v>9.12</v>
       </c>
       <c r="E106" t="str">
-        <v>贝斯旺国际有限公司</v>
+        <v>Demo Merchant West Inc.</v>
       </c>
       <c r="F106" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G106" t="str">
         <v>退税</v>
@@ -2833,10 +2833,10 @@
         <v>9.12</v>
       </c>
       <c r="E107" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F107" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G107" t="str">
         <v>FOB</v>
@@ -2856,10 +2856,10 @@
         <v>10.27</v>
       </c>
       <c r="E108" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>Demo Trading Entity A</v>
       </c>
       <c r="F108" t="str">
-        <v>泉州恒美家居有限公司</v>
+        <v>演示工厂 C</v>
       </c>
       <c r="G108" t="str">
         <v>退税</v>
@@ -2879,10 +2879,10 @@
         <v>10.27</v>
       </c>
       <c r="E109" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F109" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G109" t="str">
         <v>FOB</v>
@@ -2902,10 +2902,10 @@
         <v>3.37</v>
       </c>
       <c r="E110" t="str">
-        <v>傲杰科技国际有限公司</v>
+        <v>Demo Merchant Ltd.</v>
       </c>
       <c r="F110" t="str">
-        <v>曹县海庆家具有限公司</v>
+        <v>演示工厂 A</v>
       </c>
       <c r="G110" t="str">
         <v>非退税</v>
@@ -2925,10 +2925,10 @@
         <v>3.37</v>
       </c>
       <c r="E111" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F111" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G111" t="str">
         <v>FOB</v>
@@ -2948,10 +2948,10 @@
         <v>4.52</v>
       </c>
       <c r="E112" t="str">
-        <v>郑州傲杰</v>
+        <v>Demo Merchant East Co.</v>
       </c>
       <c r="F112" t="str">
-        <v>厦门鹭泓森供应链有限公司</v>
+        <v>演示工厂 B</v>
       </c>
       <c r="G112" t="str">
         <v>退税</v>

</xml_diff>